<commit_message>
big-data: lab 1 part 1 done
</commit_message>
<xml_diff>
--- a/studying.xlsx
+++ b/studying.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t xml:space="preserve">Сделать</t>
   </si>
@@ -34,19 +34,22 @@
     <t xml:space="preserve">Backend</t>
   </si>
   <si>
-    <t xml:space="preserve">2-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">курс  посещаемость</t>
+    <t xml:space="preserve">3-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1, 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">курс</t>
+  </si>
+  <si>
+    <t xml:space="preserve">посещаемость</t>
   </si>
   <si>
     <t xml:space="preserve">Организации вычислений</t>
   </si>
   <si>
     <t xml:space="preserve">1-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">курс</t>
   </si>
   <si>
     <t xml:space="preserve">Computer Vision</t>
@@ -511,7 +514,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.33"/>
@@ -539,83 +542,88 @@
       <c r="B2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="6" t="n">
-        <v>1</v>
+      <c r="C2" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" display="курс"/>
-    <hyperlink ref="D4" r:id="rId2" display="moodle"/>
-    <hyperlink ref="D5" r:id="rId3" display="курс"/>
+    <hyperlink ref="D2" r:id="rId1" display="курс"/>
+    <hyperlink ref="E2" r:id="rId2" display="посещаемость"/>
+    <hyperlink ref="D3" r:id="rId3" display="курс"/>
+    <hyperlink ref="D4" r:id="rId4" display="moodle"/>
+    <hyperlink ref="D5" r:id="rId5" display="курс"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
sem 2 labs dump
</commit_message>
<xml_diff>
--- a/studying.xlsx
+++ b/studying.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
   <si>
     <t xml:space="preserve">Сделать</t>
   </si>
@@ -50,18 +50,6 @@
   </si>
   <si>
     <t xml:space="preserve">Обработка сигналов</t>
-  </si>
-  <si>
-    <t xml:space="preserve">По магистерской</t>
-  </si>
-  <si>
-    <t xml:space="preserve">текст</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Отчет по практике</t>
-  </si>
-  <si>
-    <t xml:space="preserve">отчёт</t>
   </si>
 </sst>
 </file>
@@ -545,31 +533,27 @@
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="6"/>
       <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="6"/>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0"/>
+      <c r="B5" s="0"/>
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="6"/>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0"/>
+      <c r="B6" s="0"/>
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>